<commit_message>
Departamento proyectos agregado a seeder y usuario valeria febres
</commit_message>
<xml_diff>
--- a/storage/app/templates/FORMATO ENTRADA MATERIAL.xlsx
+++ b/storage/app/templates/FORMATO ENTRADA MATERIAL.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADVX~1\AppData\Roaming\MobaXterm\slash\mx86_64b\RemoteFiles\67092_2_0\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADVX~1\AppData\Roaming\MobaXterm\slash\mx86_64b\RemoteFiles\66732_2_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52A2DB5F-3498-4D88-9B5B-289CE6679521}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25C3459E-830B-4EA4-8474-2E7D50B7D53F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{7B1B6560-6531-424A-94B5-F8CBA6ECCE85}"/>
   </bookViews>
@@ -461,6 +461,93 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -472,93 +559,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -965,7 +965,7 @@
   <dimension ref="A1:J42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.1796875" customWidth="1"/>
+    <col min="1" max="1" width="11.90625" customWidth="1"/>
     <col min="2" max="2" width="10.1796875" customWidth="1"/>
     <col min="3" max="3" width="7" customWidth="1"/>
     <col min="4" max="4" width="10.26953125" customWidth="1"/>
@@ -974,646 +974,646 @@
     <col min="7" max="7" width="10.54296875" customWidth="1"/>
     <col min="8" max="8" width="12.26953125" customWidth="1"/>
     <col min="9" max="9" width="13.54296875" customWidth="1"/>
-    <col min="10" max="10" width="3.81640625" customWidth="1"/>
+    <col min="10" max="10" width="5.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="38"/>
-      <c r="B1" s="38"/>
-      <c r="C1" s="40" t="s">
+      <c r="A1" s="20"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="39" t="s">
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="39"/>
+      <c r="J1" s="21"/>
     </row>
     <row r="2" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="38"/>
-      <c r="B2" s="38"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="45"/>
+      <c r="A2" s="20"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="28"/>
       <c r="I2" s="22" t="s">
         <v>2</v>
       </c>
       <c r="J2" s="22"/>
     </row>
     <row r="3" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="38"/>
-      <c r="B3" s="38"/>
-      <c r="C3" s="43"/>
-      <c r="D3" s="44"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="44"/>
-      <c r="G3" s="44"/>
-      <c r="H3" s="45"/>
+      <c r="A3" s="20"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="27"/>
+      <c r="G3" s="27"/>
+      <c r="H3" s="28"/>
       <c r="I3" s="22" t="s">
         <v>3</v>
       </c>
       <c r="J3" s="22"/>
     </row>
     <row r="4" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="38"/>
-      <c r="B4" s="38"/>
-      <c r="C4" s="43"/>
-      <c r="D4" s="44"/>
-      <c r="E4" s="44"/>
-      <c r="F4" s="44"/>
-      <c r="G4" s="44"/>
-      <c r="H4" s="45"/>
+      <c r="A4" s="20"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="28"/>
       <c r="I4" s="22" t="s">
         <v>4</v>
       </c>
       <c r="J4" s="22"/>
     </row>
     <row r="5" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="38"/>
-      <c r="B5" s="38"/>
-      <c r="C5" s="46"/>
-      <c r="D5" s="47"/>
-      <c r="E5" s="47"/>
-      <c r="F5" s="47"/>
-      <c r="G5" s="47"/>
-      <c r="H5" s="48"/>
-      <c r="I5" s="37" t="s">
+      <c r="A5" s="20"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="31"/>
+      <c r="I5" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="J5" s="37"/>
+      <c r="J5" s="18"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A6" s="26"/>
-      <c r="B6" s="26"/>
-      <c r="C6" s="26"/>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
-      <c r="F6" s="26"/>
-      <c r="G6" s="26"/>
-      <c r="H6" s="26"/>
-      <c r="I6" s="26"/>
-      <c r="J6" s="26"/>
+      <c r="A6" s="16"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="16"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="37" t="s">
+      <c r="B7" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="37"/>
-      <c r="D7" s="37"/>
-      <c r="E7" s="37"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="37"/>
-      <c r="I7" s="37"/>
-      <c r="J7" s="37"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="18"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A8" s="36" t="s">
+      <c r="A8" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="36"/>
-      <c r="C8" s="36"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="36"/>
-      <c r="F8" s="36"/>
-      <c r="G8" s="36"/>
-      <c r="H8" s="36"/>
-      <c r="I8" s="36"/>
-      <c r="J8" s="36"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="17"/>
     </row>
     <row r="9" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="37"/>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="37"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="18"/>
       <c r="F9" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G9" s="37"/>
-      <c r="H9" s="37"/>
+      <c r="G9" s="18"/>
+      <c r="H9" s="18"/>
       <c r="I9" s="6" t="s">
         <v>9</v>
       </c>
       <c r="J9" s="7"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A10" s="29"/>
-      <c r="B10" s="29"/>
-      <c r="C10" s="29"/>
-      <c r="D10" s="29"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="29"/>
-      <c r="G10" s="29"/>
-      <c r="H10" s="29"/>
-      <c r="I10" s="29"/>
-      <c r="J10" s="29"/>
+      <c r="A10" s="19"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="19"/>
+      <c r="I10" s="19"/>
+      <c r="J10" s="19"/>
     </row>
     <row r="11" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="17" t="s">
+      <c r="C11" s="47"/>
+      <c r="D11" s="47"/>
+      <c r="E11" s="47"/>
+      <c r="F11" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="G11" s="16" t="s">
+      <c r="G11" s="45" t="s">
         <v>13</v>
       </c>
-      <c r="H11" s="16" t="s">
+      <c r="H11" s="45" t="s">
         <v>14</v>
       </c>
-      <c r="I11" s="16" t="s">
+      <c r="I11" s="45" t="s">
         <v>15</v>
       </c>
-      <c r="J11" s="16"/>
+      <c r="J11" s="45"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A12" s="19"/>
-      <c r="B12" s="18"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="16"/>
-      <c r="I12" s="16"/>
-      <c r="J12" s="16"/>
+      <c r="A12" s="48"/>
+      <c r="B12" s="47"/>
+      <c r="C12" s="47"/>
+      <c r="D12" s="47"/>
+      <c r="E12" s="47"/>
+      <c r="F12" s="46"/>
+      <c r="G12" s="45"/>
+      <c r="H12" s="45"/>
+      <c r="I12" s="45"/>
+      <c r="J12" s="45"/>
     </row>
     <row r="13" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="20" t="s">
+      <c r="B13" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="21" t="s">
+      <c r="C13" s="32"/>
+      <c r="D13" s="32"/>
+      <c r="E13" s="32"/>
+      <c r="F13" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="G13" s="21" t="s">
+      <c r="G13" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="H13" s="21" t="s">
+      <c r="H13" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="I13" s="20" t="s">
+      <c r="I13" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="J13" s="20"/>
+      <c r="J13" s="32"/>
     </row>
     <row r="14" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="21"/>
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="21"/>
-      <c r="G14" s="21"/>
-      <c r="H14" s="21"/>
-      <c r="I14" s="20"/>
-      <c r="J14" s="20"/>
+      <c r="A14" s="33"/>
+      <c r="B14" s="32"/>
+      <c r="C14" s="32"/>
+      <c r="D14" s="32"/>
+      <c r="E14" s="32"/>
+      <c r="F14" s="33"/>
+      <c r="G14" s="33"/>
+      <c r="H14" s="33"/>
+      <c r="I14" s="32"/>
+      <c r="J14" s="32"/>
     </row>
     <row r="15" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="21" t="s">
+      <c r="A15" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="20" t="s">
+      <c r="B15" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="21" t="s">
+      <c r="C15" s="32"/>
+      <c r="D15" s="32"/>
+      <c r="E15" s="32"/>
+      <c r="F15" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="G15" s="21" t="s">
+      <c r="G15" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="H15" s="21" t="s">
+      <c r="H15" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="I15" s="20" t="s">
+      <c r="I15" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="J15" s="20"/>
+      <c r="J15" s="32"/>
     </row>
     <row r="16" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="21"/>
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="21"/>
-      <c r="H16" s="21"/>
-      <c r="I16" s="20"/>
-      <c r="J16" s="20"/>
+      <c r="A16" s="33"/>
+      <c r="B16" s="32"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="33"/>
+      <c r="H16" s="33"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="32"/>
     </row>
     <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="21" t="s">
+      <c r="A17" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="20" t="s">
+      <c r="B17" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="C17" s="20"/>
-      <c r="D17" s="20"/>
-      <c r="E17" s="20"/>
-      <c r="F17" s="21" t="s">
+      <c r="C17" s="32"/>
+      <c r="D17" s="32"/>
+      <c r="E17" s="32"/>
+      <c r="F17" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="G17" s="21" t="s">
+      <c r="G17" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="H17" s="21" t="s">
+      <c r="H17" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="I17" s="20" t="s">
+      <c r="I17" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="J17" s="20"/>
+      <c r="J17" s="32"/>
     </row>
     <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="21"/>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="20"/>
-      <c r="E18" s="20"/>
-      <c r="F18" s="21"/>
-      <c r="G18" s="21"/>
-      <c r="H18" s="21"/>
-      <c r="I18" s="20"/>
-      <c r="J18" s="20"/>
+      <c r="A18" s="33"/>
+      <c r="B18" s="32"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="32"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="33"/>
+      <c r="H18" s="33"/>
+      <c r="I18" s="32"/>
+      <c r="J18" s="32"/>
     </row>
     <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="21" t="s">
+      <c r="A19" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="B19" s="20" t="s">
+      <c r="B19" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="21" t="s">
+      <c r="C19" s="32"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="G19" s="21" t="s">
+      <c r="G19" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="H19" s="21" t="s">
+      <c r="H19" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="I19" s="20" t="s">
+      <c r="I19" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="J19" s="20"/>
+      <c r="J19" s="32"/>
     </row>
     <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="21"/>
-      <c r="B20" s="20"/>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20"/>
-      <c r="E20" s="20"/>
-      <c r="F20" s="21"/>
-      <c r="G20" s="21"/>
-      <c r="H20" s="21"/>
-      <c r="I20" s="20"/>
-      <c r="J20" s="20"/>
+      <c r="A20" s="33"/>
+      <c r="B20" s="32"/>
+      <c r="C20" s="32"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="33"/>
+      <c r="G20" s="33"/>
+      <c r="H20" s="33"/>
+      <c r="I20" s="32"/>
+      <c r="J20" s="32"/>
     </row>
     <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="20" t="s">
+      <c r="B21" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="C21" s="20"/>
-      <c r="D21" s="20"/>
-      <c r="E21" s="20"/>
-      <c r="F21" s="21" t="s">
+      <c r="C21" s="32"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="G21" s="21" t="s">
+      <c r="G21" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="H21" s="21" t="s">
+      <c r="H21" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="I21" s="20" t="s">
+      <c r="I21" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="J21" s="20"/>
+      <c r="J21" s="32"/>
     </row>
     <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="21"/>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
-      <c r="D22" s="20"/>
-      <c r="E22" s="20"/>
-      <c r="F22" s="21"/>
-      <c r="G22" s="21"/>
-      <c r="H22" s="21"/>
-      <c r="I22" s="20"/>
-      <c r="J22" s="20"/>
+      <c r="A22" s="33"/>
+      <c r="B22" s="32"/>
+      <c r="C22" s="32"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="32"/>
+      <c r="J22" s="32"/>
     </row>
     <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="21" t="s">
+      <c r="A23" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="B23" s="20" t="s">
+      <c r="B23" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="C23" s="20"/>
-      <c r="D23" s="20"/>
-      <c r="E23" s="20"/>
-      <c r="F23" s="21" t="s">
+      <c r="C23" s="32"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="32"/>
+      <c r="F23" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="G23" s="21" t="s">
+      <c r="G23" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="H23" s="21" t="s">
+      <c r="H23" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="I23" s="20" t="s">
+      <c r="I23" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="J23" s="20"/>
+      <c r="J23" s="32"/>
     </row>
     <row r="24" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="21"/>
-      <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
-      <c r="D24" s="20"/>
-      <c r="E24" s="20"/>
-      <c r="F24" s="21"/>
-      <c r="G24" s="21"/>
-      <c r="H24" s="21"/>
-      <c r="I24" s="20"/>
-      <c r="J24" s="20"/>
+      <c r="A24" s="33"/>
+      <c r="B24" s="32"/>
+      <c r="C24" s="32"/>
+      <c r="D24" s="32"/>
+      <c r="E24" s="32"/>
+      <c r="F24" s="33"/>
+      <c r="G24" s="33"/>
+      <c r="H24" s="33"/>
+      <c r="I24" s="32"/>
+      <c r="J24" s="32"/>
     </row>
     <row r="25" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="21" t="s">
+      <c r="A25" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="B25" s="20" t="s">
+      <c r="B25" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="C25" s="20"/>
-      <c r="D25" s="20"/>
-      <c r="E25" s="20"/>
-      <c r="F25" s="21" t="s">
+      <c r="C25" s="32"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="32"/>
+      <c r="F25" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="G25" s="21" t="s">
+      <c r="G25" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="H25" s="21" t="s">
+      <c r="H25" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="I25" s="20" t="s">
+      <c r="I25" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="J25" s="20"/>
+      <c r="J25" s="32"/>
     </row>
     <row r="26" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="21"/>
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
-      <c r="D26" s="20"/>
-      <c r="E26" s="20"/>
-      <c r="F26" s="21"/>
-      <c r="G26" s="21"/>
-      <c r="H26" s="21"/>
-      <c r="I26" s="20"/>
-      <c r="J26" s="20"/>
+      <c r="A26" s="33"/>
+      <c r="B26" s="32"/>
+      <c r="C26" s="32"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="32"/>
+      <c r="F26" s="33"/>
+      <c r="G26" s="33"/>
+      <c r="H26" s="33"/>
+      <c r="I26" s="32"/>
+      <c r="J26" s="32"/>
     </row>
     <row r="27" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="21" t="s">
+      <c r="A27" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="B27" s="20" t="s">
+      <c r="B27" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="C27" s="20"/>
-      <c r="D27" s="20"/>
-      <c r="E27" s="20"/>
-      <c r="F27" s="21" t="s">
+      <c r="C27" s="32"/>
+      <c r="D27" s="32"/>
+      <c r="E27" s="32"/>
+      <c r="F27" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="G27" s="21" t="s">
+      <c r="G27" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="H27" s="21" t="s">
+      <c r="H27" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="I27" s="20" t="s">
+      <c r="I27" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="J27" s="20"/>
+      <c r="J27" s="32"/>
     </row>
     <row r="28" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="21"/>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
-      <c r="D28" s="20"/>
-      <c r="E28" s="20"/>
-      <c r="F28" s="21"/>
-      <c r="G28" s="21"/>
-      <c r="H28" s="21"/>
-      <c r="I28" s="20"/>
-      <c r="J28" s="20"/>
+      <c r="A28" s="33"/>
+      <c r="B28" s="32"/>
+      <c r="C28" s="32"/>
+      <c r="D28" s="32"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="33"/>
+      <c r="G28" s="33"/>
+      <c r="H28" s="33"/>
+      <c r="I28" s="32"/>
+      <c r="J28" s="32"/>
     </row>
     <row r="29" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="21" t="s">
+      <c r="A29" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="B29" s="20" t="s">
+      <c r="B29" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="C29" s="20"/>
-      <c r="D29" s="20"/>
-      <c r="E29" s="20"/>
-      <c r="F29" s="21" t="s">
+      <c r="C29" s="32"/>
+      <c r="D29" s="32"/>
+      <c r="E29" s="32"/>
+      <c r="F29" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="G29" s="21" t="s">
+      <c r="G29" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="H29" s="21" t="s">
+      <c r="H29" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="I29" s="20" t="s">
+      <c r="I29" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="J29" s="20"/>
+      <c r="J29" s="32"/>
     </row>
     <row r="30" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="21"/>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="20"/>
-      <c r="E30" s="20"/>
-      <c r="F30" s="21"/>
-      <c r="G30" s="21"/>
-      <c r="H30" s="21"/>
-      <c r="I30" s="20"/>
-      <c r="J30" s="20"/>
+      <c r="A30" s="33"/>
+      <c r="B30" s="32"/>
+      <c r="C30" s="32"/>
+      <c r="D30" s="32"/>
+      <c r="E30" s="32"/>
+      <c r="F30" s="33"/>
+      <c r="G30" s="33"/>
+      <c r="H30" s="33"/>
+      <c r="I30" s="32"/>
+      <c r="J30" s="32"/>
     </row>
     <row r="31" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="21" t="s">
+      <c r="A31" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="B31" s="20" t="s">
+      <c r="B31" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="C31" s="20"/>
-      <c r="D31" s="20"/>
-      <c r="E31" s="20"/>
-      <c r="F31" s="21" t="s">
+      <c r="C31" s="32"/>
+      <c r="D31" s="32"/>
+      <c r="E31" s="32"/>
+      <c r="F31" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="G31" s="21" t="s">
+      <c r="G31" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="H31" s="21" t="s">
+      <c r="H31" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="I31" s="20" t="s">
+      <c r="I31" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="J31" s="20"/>
+      <c r="J31" s="32"/>
     </row>
     <row r="32" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="21"/>
-      <c r="B32" s="20"/>
-      <c r="C32" s="20"/>
-      <c r="D32" s="20"/>
-      <c r="E32" s="20"/>
-      <c r="F32" s="21"/>
-      <c r="G32" s="21"/>
-      <c r="H32" s="21"/>
-      <c r="I32" s="20"/>
-      <c r="J32" s="20"/>
+      <c r="A32" s="33"/>
+      <c r="B32" s="32"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="33"/>
+      <c r="G32" s="33"/>
+      <c r="H32" s="33"/>
+      <c r="I32" s="32"/>
+      <c r="J32" s="32"/>
     </row>
     <row r="33" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="21" t="s">
+      <c r="A33" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="B33" s="20" t="s">
+      <c r="B33" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="C33" s="20"/>
-      <c r="D33" s="20"/>
-      <c r="E33" s="20"/>
-      <c r="F33" s="21" t="s">
+      <c r="C33" s="32"/>
+      <c r="D33" s="32"/>
+      <c r="E33" s="32"/>
+      <c r="F33" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="G33" s="21" t="s">
+      <c r="G33" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="H33" s="21" t="s">
+      <c r="H33" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="I33" s="20" t="s">
+      <c r="I33" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="J33" s="20"/>
+      <c r="J33" s="32"/>
     </row>
     <row r="34" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="21"/>
-      <c r="B34" s="20"/>
-      <c r="C34" s="20"/>
-      <c r="D34" s="20"/>
-      <c r="E34" s="20"/>
-      <c r="F34" s="21"/>
-      <c r="G34" s="21"/>
-      <c r="H34" s="21"/>
-      <c r="I34" s="20"/>
-      <c r="J34" s="20"/>
+      <c r="A34" s="33"/>
+      <c r="B34" s="32"/>
+      <c r="C34" s="32"/>
+      <c r="D34" s="32"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="33"/>
+      <c r="G34" s="33"/>
+      <c r="H34" s="33"/>
+      <c r="I34" s="32"/>
+      <c r="J34" s="32"/>
     </row>
     <row r="35" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="21" t="s">
+      <c r="A35" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="B35" s="20" t="s">
+      <c r="B35" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="C35" s="20"/>
-      <c r="D35" s="20"/>
-      <c r="E35" s="20"/>
-      <c r="F35" s="21" t="s">
+      <c r="C35" s="32"/>
+      <c r="D35" s="32"/>
+      <c r="E35" s="32"/>
+      <c r="F35" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="G35" s="21" t="s">
+      <c r="G35" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="H35" s="21" t="s">
+      <c r="H35" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="I35" s="20" t="s">
+      <c r="I35" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="J35" s="20"/>
+      <c r="J35" s="32"/>
     </row>
     <row r="36" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="21"/>
-      <c r="B36" s="20"/>
-      <c r="C36" s="20"/>
-      <c r="D36" s="20"/>
-      <c r="E36" s="20"/>
-      <c r="F36" s="21"/>
-      <c r="G36" s="21"/>
-      <c r="H36" s="21"/>
-      <c r="I36" s="20"/>
-      <c r="J36" s="20"/>
+      <c r="A36" s="33"/>
+      <c r="B36" s="32"/>
+      <c r="C36" s="32"/>
+      <c r="D36" s="32"/>
+      <c r="E36" s="32"/>
+      <c r="F36" s="33"/>
+      <c r="G36" s="33"/>
+      <c r="H36" s="33"/>
+      <c r="I36" s="32"/>
+      <c r="J36" s="32"/>
     </row>
     <row r="37" spans="1:10" ht="38.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="29" t="s">
+      <c r="A37" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="B37" s="29"/>
-      <c r="C37" s="31" t="s">
+      <c r="B37" s="19"/>
+      <c r="C37" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="D37" s="32"/>
-      <c r="E37" s="32"/>
-      <c r="F37" s="32"/>
-      <c r="G37" s="32"/>
-      <c r="H37" s="32"/>
-      <c r="I37" s="32"/>
-      <c r="J37" s="33"/>
+      <c r="D37" s="41"/>
+      <c r="E37" s="41"/>
+      <c r="F37" s="41"/>
+      <c r="G37" s="41"/>
+      <c r="H37" s="41"/>
+      <c r="I37" s="41"/>
+      <c r="J37" s="42"/>
     </row>
     <row r="38" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="29" t="s">
+      <c r="A38" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="B38" s="29"/>
-      <c r="C38" s="34" t="s">
+      <c r="B38" s="19"/>
+      <c r="C38" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="D38" s="35"/>
+      <c r="D38" s="44"/>
       <c r="E38" s="1" t="s">
         <v>19</v>
       </c>
@@ -1626,10 +1626,10 @@
       <c r="H38" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I38" s="30" t="s">
+      <c r="I38" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="J38" s="30"/>
+      <c r="J38" s="39"/>
     </row>
     <row r="39" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="22" t="s">
@@ -1639,13 +1639,13 @@
       <c r="C39" s="22"/>
       <c r="D39" s="22"/>
       <c r="E39" s="22"/>
-      <c r="F39" s="26" t="s">
+      <c r="F39" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="G39" s="26"/>
-      <c r="H39" s="26"/>
-      <c r="I39" s="26"/>
-      <c r="J39" s="26"/>
+      <c r="G39" s="16"/>
+      <c r="H39" s="16"/>
+      <c r="I39" s="16"/>
+      <c r="J39" s="16"/>
     </row>
     <row r="40" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="22" t="s">
@@ -1657,19 +1657,19 @@
         <v>37</v>
       </c>
       <c r="E40" s="4"/>
-      <c r="F40" s="27" t="s">
+      <c r="F40" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="G40" s="27"/>
-      <c r="H40" s="27"/>
-      <c r="I40" s="27"/>
-      <c r="J40" s="27"/>
+      <c r="G40" s="37"/>
+      <c r="H40" s="37"/>
+      <c r="I40" s="37"/>
+      <c r="J40" s="37"/>
     </row>
     <row r="41" spans="1:10" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="28" t="s">
+      <c r="A41" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="B41" s="28"/>
+      <c r="B41" s="38"/>
       <c r="C41" s="9"/>
       <c r="D41" s="10"/>
       <c r="E41" s="11"/>
@@ -1688,89 +1688,28 @@
         <v>29</v>
       </c>
       <c r="E42" s="3"/>
-      <c r="F42" s="23" t="s">
+      <c r="F42" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G42" s="24"/>
-      <c r="H42" s="24"/>
-      <c r="I42" s="24"/>
-      <c r="J42" s="25"/>
+      <c r="G42" s="35"/>
+      <c r="H42" s="35"/>
+      <c r="I42" s="35"/>
+      <c r="J42" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="103">
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="A10:J10"/>
-    <mergeCell ref="A1:B5"/>
-    <mergeCell ref="I1:J1"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="B7:J7"/>
-    <mergeCell ref="C1:H5"/>
-    <mergeCell ref="I17:J18"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="B15:E16"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="H15:H16"/>
-    <mergeCell ref="H19:H20"/>
-    <mergeCell ref="I19:J20"/>
-    <mergeCell ref="H17:H18"/>
-    <mergeCell ref="G17:G18"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="B17:E18"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="I15:J16"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="B21:E22"/>
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="G21:G22"/>
-    <mergeCell ref="H21:H22"/>
-    <mergeCell ref="I21:J22"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="B19:E20"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="H23:H24"/>
-    <mergeCell ref="I23:J24"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="B25:E26"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="G25:G26"/>
-    <mergeCell ref="H25:H26"/>
-    <mergeCell ref="I25:J26"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="B23:E24"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="G23:G24"/>
-    <mergeCell ref="H27:H28"/>
-    <mergeCell ref="I27:J28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="B29:E30"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="G29:G30"/>
-    <mergeCell ref="H29:H30"/>
-    <mergeCell ref="I29:J30"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="B27:E28"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="G27:G28"/>
-    <mergeCell ref="H31:H32"/>
-    <mergeCell ref="I31:J32"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="B33:E34"/>
-    <mergeCell ref="F33:F34"/>
-    <mergeCell ref="G33:G34"/>
-    <mergeCell ref="H33:H34"/>
-    <mergeCell ref="I33:J34"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="B31:E32"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="G31:G32"/>
+    <mergeCell ref="I11:J12"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="B11:E12"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="I13:J14"/>
+    <mergeCell ref="H13:H14"/>
+    <mergeCell ref="G13:G14"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="B13:E14"/>
+    <mergeCell ref="A13:A14"/>
     <mergeCell ref="A42:B42"/>
     <mergeCell ref="F42:J42"/>
     <mergeCell ref="A39:E39"/>
@@ -1789,22 +1728,83 @@
     <mergeCell ref="G35:G36"/>
     <mergeCell ref="C37:J37"/>
     <mergeCell ref="C38:D38"/>
-    <mergeCell ref="I11:J12"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="B11:E12"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="I13:J14"/>
-    <mergeCell ref="H13:H14"/>
-    <mergeCell ref="G13:G14"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="B13:E14"/>
-    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="H31:H32"/>
+    <mergeCell ref="I31:J32"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="B33:E34"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="G33:G34"/>
+    <mergeCell ref="H33:H34"/>
+    <mergeCell ref="I33:J34"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="B31:E32"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="G31:G32"/>
+    <mergeCell ref="H27:H28"/>
+    <mergeCell ref="I27:J28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="B29:E30"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="G29:G30"/>
+    <mergeCell ref="H29:H30"/>
+    <mergeCell ref="I29:J30"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="B27:E28"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="G27:G28"/>
+    <mergeCell ref="H23:H24"/>
+    <mergeCell ref="I23:J24"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="B25:E26"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="H25:H26"/>
+    <mergeCell ref="I25:J26"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="B23:E24"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="G23:G24"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:E22"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="H21:H22"/>
+    <mergeCell ref="I21:J22"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="B19:E20"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="I17:J18"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="B15:E16"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="H15:H16"/>
+    <mergeCell ref="H19:H20"/>
+    <mergeCell ref="I19:J20"/>
+    <mergeCell ref="H17:H18"/>
+    <mergeCell ref="G17:G18"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="B17:E18"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="I15:J16"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="A10:J10"/>
+    <mergeCell ref="A1:B5"/>
+    <mergeCell ref="I1:J1"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="B7:J7"/>
+    <mergeCell ref="C1:H5"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup scale="92" orientation="portrait" r:id="rId1"/>
+  <pageSetup scale="90" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>